<commit_message>
final 4th sheet added
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/certificates data.xlsx
+++ b/certificates data.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="1"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="1" sheetId="1" state="visible" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2912" uniqueCount="2912">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2913" uniqueCount="2913">
   <si>
     <t xml:space="preserve">Program Name</t>
   </si>
@@ -8743,6 +8743,9 @@
   </si>
   <si>
     <t>https://drive.google.com/file/d/17aUuH1zh2QFm_baUArun_GgIrWADaZnP/view?usp=drivesdk</t>
+  </si>
+  <si>
+    <t>PIA</t>
   </si>
   <si>
     <t xml:space="preserve">Dr Nirav, </t>
@@ -9293,7 +9296,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="71">
+  <borders count="70">
     <border>
       <left style="none"/>
       <right style="none"/>
@@ -10239,21 +10242,6 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FF442F65"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFF8F9FA"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFCCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="2"/>
-      </bottom>
-      <diagonal style="none"/>
-    </border>
-    <border>
-      <left style="thin">
         <color rgb="FFCCCCCC"/>
       </left>
       <right style="none"/>
@@ -10269,7 +10257,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="404">
+  <cellXfs count="406">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment readingOrder="0"/>
     </xf>
@@ -11355,46 +11343,52 @@
     <xf fontId="34" fillId="6" borderId="25" numFmtId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" readingOrder="0" vertical="center" wrapText="1"/>
     </xf>
+    <xf fontId="35" fillId="6" borderId="24" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="50" fillId="4" borderId="31" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" readingOrder="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="33" fillId="4" borderId="31" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="34" fillId="4" borderId="31" numFmtId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" readingOrder="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="50" fillId="6" borderId="36" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" readingOrder="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="33" fillId="6" borderId="36" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="34" fillId="6" borderId="36" numFmtId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" readingOrder="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="33" fillId="6" borderId="67" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" readingOrder="0" vertical="center" wrapText="1"/>
+    </xf>
     <xf fontId="0" fillId="4" borderId="30" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" readingOrder="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="50" fillId="4" borderId="31" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="50" fillId="4" borderId="68" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" readingOrder="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="33" fillId="4" borderId="31" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="34" fillId="4" borderId="31" numFmtId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" readingOrder="0" vertical="center" wrapText="1"/>
+    <xf fontId="0" fillId="4" borderId="30" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="50" fillId="6" borderId="68" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" readingOrder="0" vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="6" borderId="39" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" readingOrder="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="50" fillId="6" borderId="36" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" readingOrder="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="33" fillId="6" borderId="36" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="34" fillId="6" borderId="36" numFmtId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" readingOrder="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="33" fillId="6" borderId="67" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" readingOrder="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="50" fillId="4" borderId="68" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" readingOrder="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="50" fillId="6" borderId="68" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" readingOrder="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="6" borderId="69" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" readingOrder="0" vertical="center" wrapText="1"/>
+    <xf fontId="0" fillId="6" borderId="39" numFmtId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="50" fillId="6" borderId="48" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" readingOrder="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf fontId="50" fillId="6" borderId="70" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf fontId="50" fillId="6" borderId="69" numFmtId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" readingOrder="0" vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="34" fillId="6" borderId="48" numFmtId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -27537,7 +27531,9 @@
       <c r="N2" s="190"/>
     </row>
     <row r="3" ht="25.5" customHeight="1">
-      <c r="A3" s="389"/>
+      <c r="A3" s="389" t="s">
+        <v>2707</v>
+      </c>
       <c r="B3" s="390" t="s">
         <v>2716</v>
       </c>
@@ -27575,26 +27571,28 @@
       <c r="N3" s="190"/>
     </row>
     <row r="4" ht="25.5" customHeight="1">
-      <c r="A4" s="393"/>
-      <c r="B4" s="394" t="s">
+      <c r="A4" s="389" t="s">
+        <v>2707</v>
+      </c>
+      <c r="B4" s="393" t="s">
         <v>2723</v>
       </c>
-      <c r="C4" s="394" t="s">
+      <c r="C4" s="393" t="s">
         <v>2724</v>
       </c>
-      <c r="D4" s="394" t="s">
+      <c r="D4" s="393" t="s">
         <v>2725</v>
       </c>
-      <c r="E4" s="394" t="s">
+      <c r="E4" s="393" t="s">
         <v>2726</v>
       </c>
       <c r="F4" s="203" t="s">
         <v>2727</v>
       </c>
-      <c r="G4" s="395" t="s">
+      <c r="G4" s="394" t="s">
         <v>1520</v>
       </c>
-      <c r="H4" s="396">
+      <c r="H4" s="395">
         <v>46139</v>
       </c>
       <c r="I4" s="203" t="s">
@@ -27613,7 +27611,9 @@
       <c r="N4" s="190"/>
     </row>
     <row r="5" ht="25.5" customHeight="1">
-      <c r="A5" s="389"/>
+      <c r="A5" s="389" t="s">
+        <v>2707</v>
+      </c>
       <c r="B5" s="390" t="s">
         <v>2731</v>
       </c>
@@ -27651,26 +27651,28 @@
       <c r="N5" s="190"/>
     </row>
     <row r="6" ht="25.5" customHeight="1">
-      <c r="A6" s="393"/>
-      <c r="B6" s="394" t="s">
+      <c r="A6" s="389" t="s">
+        <v>2707</v>
+      </c>
+      <c r="B6" s="393" t="s">
         <v>2738</v>
       </c>
-      <c r="C6" s="394" t="s">
+      <c r="C6" s="393" t="s">
         <v>2739</v>
       </c>
-      <c r="D6" s="394" t="s">
+      <c r="D6" s="393" t="s">
         <v>2740</v>
       </c>
-      <c r="E6" s="394" t="s">
+      <c r="E6" s="393" t="s">
         <v>2741</v>
       </c>
       <c r="F6" s="203" t="s">
         <v>2742</v>
       </c>
-      <c r="G6" s="395" t="s">
+      <c r="G6" s="394" t="s">
         <v>1532</v>
       </c>
-      <c r="H6" s="396">
+      <c r="H6" s="395">
         <v>46139</v>
       </c>
       <c r="I6" s="203" t="s">
@@ -27689,7 +27691,9 @@
       <c r="N6" s="190"/>
     </row>
     <row r="7" ht="25.5" customHeight="1">
-      <c r="A7" s="389"/>
+      <c r="A7" s="389" t="s">
+        <v>2707</v>
+      </c>
       <c r="B7" s="390" t="s">
         <v>2745</v>
       </c>
@@ -27727,26 +27731,28 @@
       <c r="N7" s="190"/>
     </row>
     <row r="8" ht="25.5" customHeight="1">
-      <c r="A8" s="393"/>
-      <c r="B8" s="394" t="s">
+      <c r="A8" s="389" t="s">
+        <v>2707</v>
+      </c>
+      <c r="B8" s="393" t="s">
         <v>2752</v>
       </c>
-      <c r="C8" s="394" t="s">
+      <c r="C8" s="393" t="s">
         <v>2753</v>
       </c>
-      <c r="D8" s="394" t="s">
+      <c r="D8" s="393" t="s">
         <v>2754</v>
       </c>
-      <c r="E8" s="394" t="s">
+      <c r="E8" s="393" t="s">
         <v>2755</v>
       </c>
       <c r="F8" s="203" t="s">
         <v>2756</v>
       </c>
-      <c r="G8" s="395" t="s">
+      <c r="G8" s="394" t="s">
         <v>1544</v>
       </c>
-      <c r="H8" s="396">
+      <c r="H8" s="395">
         <v>46139</v>
       </c>
       <c r="I8" s="203" t="s">
@@ -27765,7 +27771,9 @@
       <c r="N8" s="190"/>
     </row>
     <row r="9" ht="25.5" customHeight="1">
-      <c r="A9" s="389"/>
+      <c r="A9" s="389" t="s">
+        <v>2707</v>
+      </c>
       <c r="B9" s="390" t="s">
         <v>2759</v>
       </c>
@@ -27803,26 +27811,28 @@
       <c r="N9" s="190"/>
     </row>
     <row r="10" ht="25.5" customHeight="1">
-      <c r="A10" s="393"/>
-      <c r="B10" s="394" t="s">
+      <c r="A10" s="389" t="s">
+        <v>2707</v>
+      </c>
+      <c r="B10" s="393" t="s">
         <v>2766</v>
       </c>
-      <c r="C10" s="394" t="s">
+      <c r="C10" s="393" t="s">
         <v>2767</v>
       </c>
-      <c r="D10" s="394" t="s">
+      <c r="D10" s="393" t="s">
         <v>2482</v>
       </c>
-      <c r="E10" s="394" t="s">
+      <c r="E10" s="393" t="s">
         <v>2768</v>
       </c>
       <c r="F10" s="203" t="s">
         <v>2769</v>
       </c>
-      <c r="G10" s="397" t="s">
+      <c r="G10" s="396" t="s">
         <v>1557</v>
       </c>
-      <c r="H10" s="396">
+      <c r="H10" s="395">
         <v>46139</v>
       </c>
       <c r="I10" s="203" t="s">
@@ -27841,7 +27851,9 @@
       <c r="N10" s="190"/>
     </row>
     <row r="11" ht="25.5" customHeight="1">
-      <c r="A11" s="389"/>
+      <c r="A11" s="397" t="s">
+        <v>1619</v>
+      </c>
       <c r="B11" s="390" t="s">
         <v>2773</v>
       </c>
@@ -27879,17 +27891,19 @@
       <c r="N11" s="190"/>
     </row>
     <row r="12" ht="25.5" customHeight="1">
-      <c r="A12" s="393"/>
-      <c r="B12" s="394" t="s">
+      <c r="A12" s="399" t="s">
+        <v>1619</v>
+      </c>
+      <c r="B12" s="393" t="s">
         <v>2781</v>
       </c>
-      <c r="C12" s="394" t="s">
+      <c r="C12" s="393" t="s">
         <v>2782</v>
       </c>
-      <c r="D12" s="399" t="s">
+      <c r="D12" s="400" t="s">
         <v>2783</v>
       </c>
-      <c r="E12" s="399" t="s">
+      <c r="E12" s="400" t="s">
         <v>2784</v>
       </c>
       <c r="F12" s="212" t="s">
@@ -27898,7 +27912,7 @@
       <c r="G12" s="194" t="s">
         <v>2786</v>
       </c>
-      <c r="H12" s="396">
+      <c r="H12" s="395">
         <v>46139</v>
       </c>
       <c r="I12" s="203" t="s">
@@ -27917,7 +27931,9 @@
       <c r="N12" s="190"/>
     </row>
     <row r="13" ht="25.5" customHeight="1">
-      <c r="A13" s="389"/>
+      <c r="A13" s="399" t="s">
+        <v>1619</v>
+      </c>
       <c r="B13" s="390" t="s">
         <v>2789</v>
       </c>
@@ -27955,17 +27971,19 @@
       <c r="N13" s="190"/>
     </row>
     <row r="14" ht="25.5" customHeight="1">
-      <c r="A14" s="393"/>
-      <c r="B14" s="394" t="s">
+      <c r="A14" s="399" t="s">
+        <v>1619</v>
+      </c>
+      <c r="B14" s="393" t="s">
         <v>2796</v>
       </c>
-      <c r="C14" s="394" t="s">
+      <c r="C14" s="393" t="s">
         <v>2797</v>
       </c>
-      <c r="D14" s="399" t="s">
+      <c r="D14" s="400" t="s">
         <v>2798</v>
       </c>
-      <c r="E14" s="399" t="s">
+      <c r="E14" s="400" t="s">
         <v>2799</v>
       </c>
       <c r="F14" s="212" t="s">
@@ -27974,7 +27992,7 @@
       <c r="G14" s="194" t="s">
         <v>2801</v>
       </c>
-      <c r="H14" s="396">
+      <c r="H14" s="395">
         <v>46139</v>
       </c>
       <c r="I14" s="203" t="s">
@@ -27993,17 +28011,19 @@
       <c r="N14" s="190"/>
     </row>
     <row r="15" ht="25.5" customHeight="1">
-      <c r="A15" s="393"/>
-      <c r="B15" s="394" t="s">
+      <c r="A15" s="399" t="s">
+        <v>1619</v>
+      </c>
+      <c r="B15" s="393" t="s">
         <v>2804</v>
       </c>
-      <c r="C15" s="394" t="s">
+      <c r="C15" s="393" t="s">
         <v>2805</v>
       </c>
-      <c r="D15" s="399" t="s">
+      <c r="D15" s="400" t="s">
         <v>2806</v>
       </c>
-      <c r="E15" s="399" t="s">
+      <c r="E15" s="400" t="s">
         <v>2807</v>
       </c>
       <c r="F15" s="212" t="s">
@@ -28012,7 +28032,7 @@
       <c r="G15" s="194" t="s">
         <v>2809</v>
       </c>
-      <c r="H15" s="396">
+      <c r="H15" s="395">
         <v>46139</v>
       </c>
       <c r="I15" s="203" t="s">
@@ -28031,7 +28051,9 @@
       <c r="N15" s="190"/>
     </row>
     <row r="16" ht="25.5" customHeight="1">
-      <c r="A16" s="389"/>
+      <c r="A16" s="399" t="s">
+        <v>1619</v>
+      </c>
       <c r="B16" s="390" t="s">
         <v>2812</v>
       </c>
@@ -28109,17 +28131,19 @@
       <c r="N17" s="190"/>
     </row>
     <row r="18" ht="25.5" customHeight="1">
-      <c r="A18" s="393"/>
-      <c r="B18" s="394" t="s">
+      <c r="A18" s="324" t="s">
+        <v>2558</v>
+      </c>
+      <c r="B18" s="393" t="s">
         <v>2829</v>
       </c>
-      <c r="C18" s="394" t="s">
+      <c r="C18" s="393" t="s">
         <v>2830</v>
       </c>
-      <c r="D18" s="399" t="s">
+      <c r="D18" s="400" t="s">
         <v>2831</v>
       </c>
-      <c r="E18" s="399" t="s">
+      <c r="E18" s="400" t="s">
         <v>2832</v>
       </c>
       <c r="F18" s="212" t="s">
@@ -28128,7 +28152,7 @@
       <c r="G18" s="194" t="s">
         <v>2834</v>
       </c>
-      <c r="H18" s="396">
+      <c r="H18" s="395">
         <v>46139</v>
       </c>
       <c r="I18" s="203" t="s">
@@ -28147,7 +28171,9 @@
       <c r="N18" s="190"/>
     </row>
     <row r="19" ht="25.5" customHeight="1">
-      <c r="A19" s="389"/>
+      <c r="A19" s="324" t="s">
+        <v>2558</v>
+      </c>
       <c r="B19" s="390" t="s">
         <v>2837</v>
       </c>
@@ -28185,17 +28211,19 @@
       <c r="N19" s="190"/>
     </row>
     <row r="20" ht="25.5" customHeight="1">
-      <c r="A20" s="393"/>
-      <c r="B20" s="394" t="s">
+      <c r="A20" s="324" t="s">
+        <v>2558</v>
+      </c>
+      <c r="B20" s="393" t="s">
         <v>2845</v>
       </c>
-      <c r="C20" s="394" t="s">
+      <c r="C20" s="393" t="s">
         <v>2846</v>
       </c>
-      <c r="D20" s="399" t="s">
+      <c r="D20" s="400" t="s">
         <v>2847</v>
       </c>
-      <c r="E20" s="399" t="s">
+      <c r="E20" s="400" t="s">
         <v>2848</v>
       </c>
       <c r="F20" s="212" t="s">
@@ -28204,7 +28232,7 @@
       <c r="G20" s="194" t="s">
         <v>2850</v>
       </c>
-      <c r="H20" s="396">
+      <c r="H20" s="395">
         <v>46139</v>
       </c>
       <c r="I20" s="203" t="s">
@@ -28223,7 +28251,9 @@
       <c r="N20" s="190"/>
     </row>
     <row r="21" ht="25.5" customHeight="1">
-      <c r="A21" s="389"/>
+      <c r="A21" s="324" t="s">
+        <v>2558</v>
+      </c>
       <c r="B21" s="390" t="s">
         <v>2854</v>
       </c>
@@ -28261,17 +28291,19 @@
       <c r="N21" s="190"/>
     </row>
     <row r="22" ht="25.5" customHeight="1">
-      <c r="A22" s="393"/>
-      <c r="B22" s="394" t="s">
+      <c r="A22" s="324" t="s">
+        <v>2558</v>
+      </c>
+      <c r="B22" s="393" t="s">
         <v>2862</v>
       </c>
-      <c r="C22" s="394" t="s">
+      <c r="C22" s="393" t="s">
         <v>2863</v>
       </c>
-      <c r="D22" s="399" t="s">
+      <c r="D22" s="400" t="s">
         <v>2864</v>
       </c>
-      <c r="E22" s="399" t="s">
+      <c r="E22" s="400" t="s">
         <v>2865</v>
       </c>
       <c r="F22" s="212" t="s">
@@ -28280,7 +28312,7 @@
       <c r="G22" s="194" t="s">
         <v>2867</v>
       </c>
-      <c r="H22" s="396">
+      <c r="H22" s="395">
         <v>46139</v>
       </c>
       <c r="I22" s="203" t="s">
@@ -28299,36 +28331,38 @@
       <c r="N22" s="190"/>
     </row>
     <row r="23" ht="25.5" customHeight="1">
-      <c r="A23" s="393"/>
-      <c r="B23" s="394" t="s">
+      <c r="A23" s="401" t="s">
         <v>2870</v>
       </c>
-      <c r="C23" s="394" t="s">
+      <c r="B23" s="393" t="s">
         <v>2871</v>
       </c>
-      <c r="D23" s="399" t="s">
+      <c r="C23" s="393" t="s">
         <v>2872</v>
       </c>
-      <c r="E23" s="399" t="s">
+      <c r="D23" s="400" t="s">
         <v>2873</v>
       </c>
+      <c r="E23" s="400" t="s">
+        <v>2874</v>
+      </c>
       <c r="F23" s="212" t="s">
-        <v>2874</v>
+        <v>2875</v>
       </c>
       <c r="G23" s="194" t="s">
         <v>1655</v>
       </c>
-      <c r="H23" s="396">
+      <c r="H23" s="395">
         <v>46139</v>
       </c>
       <c r="I23" s="203" t="s">
+        <v>2876</v>
+      </c>
+      <c r="J23" s="204" t="s">
+        <v>2877</v>
+      </c>
+      <c r="K23" s="204" t="s">
         <v>2875</v>
-      </c>
-      <c r="J23" s="204" t="s">
-        <v>2876</v>
-      </c>
-      <c r="K23" s="204" t="s">
-        <v>2874</v>
       </c>
       <c r="L23" s="205" t="s">
         <v>2295</v>
@@ -28337,36 +28371,38 @@
       <c r="N23" s="190"/>
     </row>
     <row r="24" ht="25.5" customHeight="1">
-      <c r="A24" s="389"/>
+      <c r="A24" s="402" t="s">
+        <v>2870</v>
+      </c>
       <c r="B24" s="390" t="s">
-        <v>2877</v>
+        <v>2878</v>
       </c>
       <c r="C24" s="390" t="s">
-        <v>2878</v>
+        <v>2879</v>
       </c>
       <c r="D24" s="398" t="s">
-        <v>2879</v>
+        <v>2880</v>
       </c>
       <c r="E24" s="398" t="s">
-        <v>2880</v>
+        <v>2881</v>
       </c>
       <c r="F24" s="230" t="s">
-        <v>2881</v>
+        <v>2882</v>
       </c>
       <c r="G24" s="194" t="s">
-        <v>2882</v>
+        <v>2883</v>
       </c>
       <c r="H24" s="392">
         <v>46139</v>
       </c>
       <c r="I24" s="196" t="s">
-        <v>2883</v>
+        <v>2884</v>
       </c>
       <c r="J24" s="197" t="s">
-        <v>2884</v>
+        <v>2885</v>
       </c>
       <c r="K24" s="197" t="s">
-        <v>2881</v>
+        <v>2882</v>
       </c>
       <c r="L24" s="198" t="s">
         <v>2295</v>
@@ -28375,115 +28411,121 @@
       <c r="N24" s="190"/>
     </row>
     <row r="25" ht="25.5" customHeight="1">
-      <c r="A25" s="400"/>
-      <c r="B25" s="401" t="s">
-        <v>2885</v>
-      </c>
-      <c r="C25" s="401" t="s">
+      <c r="A25" s="402" t="s">
+        <v>2870</v>
+      </c>
+      <c r="B25" s="403" t="s">
         <v>2886</v>
       </c>
-      <c r="D25" s="402" t="s">
+      <c r="C25" s="403" t="s">
         <v>2887</v>
       </c>
-      <c r="E25" s="402" t="s">
+      <c r="D25" s="404" t="s">
         <v>2888</v>
       </c>
+      <c r="E25" s="404" t="s">
+        <v>2889</v>
+      </c>
       <c r="F25" s="233" t="s">
-        <v>2889</v>
+        <v>2890</v>
       </c>
       <c r="G25" s="194" t="s">
+        <v>2891</v>
+      </c>
+      <c r="H25" s="405">
+        <v>46139</v>
+      </c>
+      <c r="I25" s="235" t="s">
+        <v>2892</v>
+      </c>
+      <c r="J25" s="236" t="s">
+        <v>2893</v>
+      </c>
+      <c r="K25" s="236" t="s">
         <v>2890</v>
       </c>
-      <c r="H25" s="403">
-        <v>46139</v>
-      </c>
-      <c r="I25" s="235" t="s">
-        <v>2891</v>
-      </c>
-      <c r="J25" s="236" t="s">
-        <v>2892</v>
-      </c>
-      <c r="K25" s="236" t="s">
-        <v>2889</v>
-      </c>
       <c r="L25" s="237" t="s">
-        <v>2893</v>
+        <v>2894</v>
       </c>
       <c r="M25" s="190"/>
       <c r="N25" s="190"/>
     </row>
     <row r="26" ht="25.5" customHeight="1">
-      <c r="A26" s="393"/>
-      <c r="B26" s="394" t="s">
-        <v>2894</v>
-      </c>
-      <c r="C26" s="394" t="s">
+      <c r="A26" s="402" t="s">
+        <v>2870</v>
+      </c>
+      <c r="B26" s="393" t="s">
         <v>2895</v>
       </c>
-      <c r="D26" s="399" t="s">
+      <c r="C26" s="393" t="s">
         <v>2896</v>
       </c>
-      <c r="E26" s="399" t="s">
+      <c r="D26" s="400" t="s">
         <v>2897</v>
       </c>
+      <c r="E26" s="400" t="s">
+        <v>2898</v>
+      </c>
       <c r="F26" s="212" t="s">
-        <v>2898</v>
+        <v>2899</v>
       </c>
       <c r="G26" s="194" t="s">
+        <v>2900</v>
+      </c>
+      <c r="H26" s="395">
+        <v>46139</v>
+      </c>
+      <c r="I26" s="203" t="s">
+        <v>2901</v>
+      </c>
+      <c r="J26" s="204" t="s">
+        <v>2902</v>
+      </c>
+      <c r="K26" s="204" t="s">
         <v>2899</v>
       </c>
-      <c r="H26" s="396">
-        <v>46139</v>
-      </c>
-      <c r="I26" s="203" t="s">
-        <v>2900</v>
-      </c>
-      <c r="J26" s="204" t="s">
-        <v>2901</v>
-      </c>
-      <c r="K26" s="204" t="s">
-        <v>2898</v>
-      </c>
       <c r="L26" s="205" t="s">
-        <v>2902</v>
+        <v>2903</v>
       </c>
       <c r="M26" s="190"/>
       <c r="N26" s="190"/>
     </row>
     <row r="27" ht="25.5" customHeight="1">
-      <c r="A27" s="389"/>
+      <c r="A27" s="402" t="s">
+        <v>2870</v>
+      </c>
       <c r="B27" s="390" t="s">
-        <v>2903</v>
+        <v>2904</v>
       </c>
       <c r="C27" s="390" t="s">
-        <v>2904</v>
+        <v>2905</v>
       </c>
       <c r="D27" s="398" t="s">
-        <v>2905</v>
+        <v>2906</v>
       </c>
       <c r="E27" s="398" t="s">
-        <v>2906</v>
+        <v>2907</v>
       </c>
       <c r="F27" s="230" t="s">
-        <v>2907</v>
+        <v>2908</v>
       </c>
       <c r="G27" s="194" t="s">
-        <v>2908</v>
+        <v>2909</v>
       </c>
       <c r="H27" s="392">
         <v>46139</v>
       </c>
       <c r="I27" s="196" t="s">
-        <v>2909</v>
+        <v>2910</v>
       </c>
       <c r="J27" s="197" t="s">
-        <v>2910</v>
+        <v>2911</v>
       </c>
       <c r="K27" s="197" t="s">
-        <v>2907</v>
+        <v>2908</v>
       </c>
       <c r="L27" s="198" t="s">
-        <v>2911</v>
+        <v>2912</v>
       </c>
       <c r="M27" s="190"/>
       <c r="N27" s="190"/>

</xml_diff>